<commit_message>
Updated Exercise 2A with AI feedback notes
</commit_message>
<xml_diff>
--- a/week-02/Ex2A_events_normalized.xlsx
+++ b/week-02/Ex2A_events_normalized.xlsx
@@ -1,22 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30611"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://reliablecollaboration.sharepoint.com/sites/Customers/Shared Documents/cust-pluralsight/YearUpSpring2026_DataAnalytics/DA course material/Week 2 - SQL Part 1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="8_{5B4E3DCD-377A-4090-B47E-5AC222FD283A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B7CB38E-A77F-49CB-8D35-7B67CF218881}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BBADFEFA-AF41-4000-8651-EA33A738C118}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1035" yWindow="630" windowWidth="38700" windowHeight="15345" xr2:uid="{5091876E-AF08-41C4-B976-D2AB9D8B455C}"/>
   </bookViews>
   <sheets>
     <sheet name="events_sample" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -33,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="178">
   <si>
     <t>Event ID</t>
   </si>
@@ -41,9 +44,51 @@
     <t>Event Name</t>
   </si>
   <si>
+    <t>Venue Location</t>
+  </si>
+  <si>
+    <t>Event Category</t>
+  </si>
+  <si>
+    <t>Category Code</t>
+  </si>
+  <si>
     <t>Event Date</t>
   </si>
   <si>
+    <t>Event Manager</t>
+  </si>
+  <si>
+    <t>Employee #</t>
+  </si>
+  <si>
+    <t>Mgr Email</t>
+  </si>
+  <si>
+    <t>Location Address</t>
+  </si>
+  <si>
+    <t>Location City</t>
+  </si>
+  <si>
+    <t>Location State</t>
+  </si>
+  <si>
+    <t>Location Zip</t>
+  </si>
+  <si>
+    <t>Venue ID</t>
+  </si>
+  <si>
+    <t>Venue Contact Name</t>
+  </si>
+  <si>
+    <t>Venue Email</t>
+  </si>
+  <si>
+    <t>Venue Phone</t>
+  </si>
+  <si>
     <t>Starlight Showcase</t>
   </si>
   <si>
@@ -56,6 +101,33 @@
     <t>Larry Song</t>
   </si>
   <si>
+    <t>u0156</t>
+  </si>
+  <si>
+    <t>larry.song@eventdoodle.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1847 Sunset Boulevard</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Los Angeles</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> CA</t>
+  </si>
+  <si>
+    <t>Starlight_CA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Maria Riley</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> maria.r@starlightbar.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (323) 555-0142</t>
+  </si>
+  <si>
     <t>Summer Jazz Festival</t>
   </si>
   <si>
@@ -65,6 +137,33 @@
     <t>Sarah Mitchell</t>
   </si>
   <si>
+    <t>u1023</t>
+  </si>
+  <si>
+    <t>sarah.mitchell@eventdoodle.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 3250 Riverside Drive</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Austin</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> TX</t>
+  </si>
+  <si>
+    <t>RivAmp_TX</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> James Mitchell</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> jmitchell@riversideamp.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (512) 555-0298</t>
+  </si>
+  <si>
     <t>Comedy Night Live</t>
   </si>
   <si>
@@ -77,6 +176,30 @@
     <t>Mike Chen</t>
   </si>
   <si>
+    <t>u0561</t>
+  </si>
+  <si>
+    <t>mike.chen@eventdoodle.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 8001 Sunset Boulevard</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> West Hollywood</t>
+  </si>
+  <si>
+    <t>LafFctry_CA</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> David Chekov</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> david@laughfactory.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (323) 555-0187</t>
+  </si>
+  <si>
     <t>Tech Innovation Summit</t>
   </si>
   <si>
@@ -86,6 +209,27 @@
     <t>Conference</t>
   </si>
   <si>
+    <t xml:space="preserve"> 1201 Convention Plaza</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Chicago</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> IL</t>
+  </si>
+  <si>
+    <t>DtwnCon_IL</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Patricia Anderson</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> p.anderson@dccchicago.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (312) 555-0456</t>
+  </si>
+  <si>
     <t>Sunset Poetry Reading</t>
   </si>
   <si>
@@ -98,6 +242,33 @@
     <t>Elena Rodriguez</t>
   </si>
   <si>
+    <t>u0865</t>
+  </si>
+  <si>
+    <t>elena.rodriguez@eventdoodle.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 428 Greenwich Avenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> New York</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> NY</t>
+  </si>
+  <si>
+    <t>CafeB_NY</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Sophie Laurent</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> sophie@cafeboheme.nyc</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (212) 555-0333</t>
+  </si>
+  <si>
     <t>Spring Food &amp; Wine Expo</t>
   </si>
   <si>
@@ -107,6 +278,12 @@
     <t>David Park</t>
   </si>
   <si>
+    <t>u0422</t>
+  </si>
+  <si>
+    <t>david.park@eventdoodle.com</t>
+  </si>
+  <si>
     <t>Indie Film Showcase</t>
   </si>
   <si>
@@ -116,6 +293,27 @@
     <t>Film</t>
   </si>
   <si>
+    <t xml:space="preserve"> 2847 Broadway Street</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Portland</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> OR</t>
+  </si>
+  <si>
+    <t>MetroCin_OR</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Robert Kim</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> robert.kim@metrocinema.org</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (503) 555-0721</t>
+  </si>
+  <si>
     <t>Corporate Leadership Forum</t>
   </si>
   <si>
@@ -125,6 +323,33 @@
     <t>Jennifer Wu</t>
   </si>
   <si>
+    <t>u0187</t>
+  </si>
+  <si>
+    <t>jennifer.wu@eventdoodle.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 500 Michigan Avenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Detroit</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> MI</t>
+  </si>
+  <si>
+    <t>GrBall_MI</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Elizabeth Thompson</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ethompson@grandballroom.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (313) 555-0892</t>
+  </si>
+  <si>
     <t>Blues &amp; BBQ Night</t>
   </si>
   <si>
@@ -134,6 +359,21 @@
     <t>Comedy Corner Club</t>
   </si>
   <si>
+    <t xml:space="preserve"> 156 Bleecker Street</t>
+  </si>
+  <si>
+    <t>ComCor_NY</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Michael O'Brien</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> mike@comedycorner.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> (212) 555-0654</t>
+  </si>
+  <si>
     <t>Art Walk Opening</t>
   </si>
   <si>
@@ -143,150 +383,6 @@
     <t>Art</t>
   </si>
   <si>
-    <t>larry.song@eventdoodle.com</t>
-  </si>
-  <si>
-    <t>sarah.mitchell@eventdoodle.com</t>
-  </si>
-  <si>
-    <t>mike.chen@eventdoodle.com</t>
-  </si>
-  <si>
-    <t>elena.rodriguez@eventdoodle.com</t>
-  </si>
-  <si>
-    <t>david.park@eventdoodle.com</t>
-  </si>
-  <si>
-    <t>jennifer.wu@eventdoodle.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1847 Sunset Boulevard</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Los Angeles</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> CA</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> maria.r@starlightbar.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> (323) 555-0142</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 3250 Riverside Drive</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Austin</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> TX</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> James Mitchell</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> jmitchell@riversideamp.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> (512) 555-0298</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 8001 Sunset Boulevard</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> West Hollywood</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> david@laughfactory.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> (323) 555-0187</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1201 Convention Plaza</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Chicago</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> IL</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Patricia Anderson</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> p.anderson@dccchicago.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> (312) 555-0456</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 428 Greenwich Avenue</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> New York</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> NY</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Sophie Laurent</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> sophie@cafeboheme.nyc</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> (212) 555-0333</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 2847 Broadway Street</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Portland</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> OR</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Robert Kim</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> robert.kim@metrocinema.org</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> (503) 555-0721</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 500 Michigan Avenue</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Detroit</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> MI</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Elizabeth Thompson</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ethompson@grandballroom.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> (313) 555-0892</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 156 Bleecker Street</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> mike@comedycorner.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> (212) 555-0654</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 975 Art Walk Lane</t>
   </si>
   <si>
@@ -296,6 +392,9 @@
     <t xml:space="preserve"> FL</t>
   </si>
   <si>
+    <t>GallDst_FL</t>
+  </si>
+  <si>
     <t xml:space="preserve"> Amanda Rivera</t>
   </si>
   <si>
@@ -305,119 +404,182 @@
     <t xml:space="preserve"> (305) 555-0401</t>
   </si>
   <si>
-    <t>Location Address</t>
-  </si>
-  <si>
-    <t>Location City</t>
-  </si>
-  <si>
-    <t>Location State</t>
-  </si>
-  <si>
-    <t>Location Zip</t>
-  </si>
-  <si>
-    <t>Venue Email</t>
-  </si>
-  <si>
-    <t>Venue Phone</t>
-  </si>
-  <si>
-    <t>Venue Contact Name</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Michael O'Brien</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Maria Riley</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> David Chekov</t>
-  </si>
-  <si>
-    <t>1st table:</t>
-  </si>
-  <si>
-    <t>2nd table:</t>
-  </si>
-  <si>
-    <t>3rd table:</t>
-  </si>
-  <si>
-    <t>Event Category</t>
-  </si>
-  <si>
-    <t>Category Code</t>
-  </si>
-  <si>
-    <t>Event Manager</t>
-  </si>
-  <si>
-    <t>Mgr Email</t>
-  </si>
-  <si>
-    <t>Employee #</t>
-  </si>
-  <si>
-    <t>u0156</t>
-  </si>
-  <si>
-    <t>u1023</t>
-  </si>
-  <si>
-    <t>u0561</t>
-  </si>
-  <si>
-    <t>u0422</t>
-  </si>
-  <si>
-    <t>u0187</t>
-  </si>
-  <si>
-    <t>Venue Location</t>
-  </si>
-  <si>
-    <t>Venue ID</t>
-  </si>
-  <si>
-    <t>RivAmp_TX</t>
-  </si>
-  <si>
-    <t>Starlight_CA</t>
-  </si>
-  <si>
-    <t>LafFctry_CA</t>
-  </si>
-  <si>
-    <t>DtwnCon_IL</t>
-  </si>
-  <si>
-    <t>CafeB_NY</t>
-  </si>
-  <si>
-    <t>MetroCin_OR</t>
-  </si>
-  <si>
-    <t>GrBall_MI</t>
-  </si>
-  <si>
-    <t>ComCor_NY</t>
-  </si>
-  <si>
-    <t>GallDst_FL</t>
-  </si>
-  <si>
-    <t>4th table?</t>
-  </si>
-  <si>
-    <t>u0865</t>
+    <t>Event Categories</t>
+  </si>
+  <si>
+    <t>Event Managers</t>
+  </si>
+  <si>
+    <t>Venues</t>
+  </si>
+  <si>
+    <t>428 Greenwich Avenue</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>NY</t>
+  </si>
+  <si>
+    <t>Sophie Laurent</t>
+  </si>
+  <si>
+    <t>sophie@cafeboheme.nyc</t>
+  </si>
+  <si>
+    <t>(212) 555-0333</t>
+  </si>
+  <si>
+    <t>156 Bleecker Street</t>
+  </si>
+  <si>
+    <t>Michael O'Brien</t>
+  </si>
+  <si>
+    <t>mike@comedycorner.com</t>
+  </si>
+  <si>
+    <t>(212) 555-0654</t>
+  </si>
+  <si>
+    <t>1201 Convention Plaza</t>
+  </si>
+  <si>
+    <t>Chicago</t>
+  </si>
+  <si>
+    <t>IL</t>
+  </si>
+  <si>
+    <t>Patricia Anderson</t>
+  </si>
+  <si>
+    <t>p.anderson@dccchicago.com</t>
+  </si>
+  <si>
+    <t>(312) 555-0456</t>
+  </si>
+  <si>
+    <t>975 Art Walk Lane</t>
+  </si>
+  <si>
+    <t>Miami</t>
+  </si>
+  <si>
+    <t>FL</t>
+  </si>
+  <si>
+    <t>Amanda Rivera</t>
+  </si>
+  <si>
+    <t>arivera@gallerydistrict.org</t>
+  </si>
+  <si>
+    <t>(305) 555-0401</t>
+  </si>
+  <si>
+    <t>500 Michigan Avenue</t>
+  </si>
+  <si>
+    <t>Detroit</t>
+  </si>
+  <si>
+    <t>MI</t>
+  </si>
+  <si>
+    <t>Elizabeth Thompson</t>
+  </si>
+  <si>
+    <t>ethompson@grandballroom.com</t>
+  </si>
+  <si>
+    <t>(313) 555-0892</t>
+  </si>
+  <si>
+    <t>8001 Sunset Boulevard</t>
+  </si>
+  <si>
+    <t>West Hollywood</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>David Chekov</t>
+  </si>
+  <si>
+    <t>david@laughfactory.com</t>
+  </si>
+  <si>
+    <t>(323) 555-0187</t>
+  </si>
+  <si>
+    <t>2847 Broadway Street</t>
+  </si>
+  <si>
+    <t>Portland</t>
+  </si>
+  <si>
+    <t>OR</t>
+  </si>
+  <si>
+    <t>Robert Kim</t>
+  </si>
+  <si>
+    <t>robert.kim@metrocinema.org</t>
+  </si>
+  <si>
+    <t>(503) 555-0721</t>
+  </si>
+  <si>
+    <t>3250 Riverside Drive</t>
+  </si>
+  <si>
+    <t>Austin</t>
+  </si>
+  <si>
+    <t>TX</t>
+  </si>
+  <si>
+    <t>James Mitchell</t>
+  </si>
+  <si>
+    <t>jmitchell@riversideamp.com</t>
+  </si>
+  <si>
+    <t>(512) 555-0298</t>
+  </si>
+  <si>
+    <t>1847 Sunset Boulevard</t>
+  </si>
+  <si>
+    <t>Los Angeles</t>
+  </si>
+  <si>
+    <t>Maria Riley</t>
+  </si>
+  <si>
+    <t>maria.r@starlightbar.com</t>
+  </si>
+  <si>
+    <t>(323) 555-0142</t>
+  </si>
+  <si>
+    <t>Events</t>
+  </si>
+  <si>
+    <t>AI feedback: Helpful that it confirmed my tables and foreign keys are correct. Splitting City/State out by ZIP and making a separate Contacts table could be more normalized, but that seems like more than this small sample needs.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="00000"/>
+  </numFmts>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -552,8 +714,24 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF7F6000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -735,7 +913,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF44546A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF4472C4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -909,12 +1099,31 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="35" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -960,7 +1169,160 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="30">
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF44546A"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="00000"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF44546A"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border>
+        <bottom style="thin">
+          <color rgb="FFD9E2F3"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -971,6 +1333,62 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2AC1FA0C-00AF-4B52-A9B5-4ACC01832871}" name="EventCategories" displayName="EventCategories" ref="A17:B24" totalsRowShown="0" dataDxfId="29" tableBorderDxfId="28">
+  <autoFilter ref="A17:B24" xr:uid="{2AC1FA0C-00AF-4B52-A9B5-4ACC01832871}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{4C44F813-D7D1-474C-8271-F54A773BC8F4}" name="Category Code" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{11181DB6-D2CE-468A-815E-35B9AF7729AB}" name="Event Category" dataDxfId="26"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{2FB88B7F-08A9-471B-BB55-BBFC8EA112C6}" name="EventManagers" displayName="EventManagers" ref="A34:C40" totalsRowShown="0" dataDxfId="25" tableBorderDxfId="24">
+  <autoFilter ref="A34:C40" xr:uid="{2FB88B7F-08A9-471B-BB55-BBFC8EA112C6}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{D0F26E47-D330-49B3-BEF2-A5DF81F48C87}" name="Employee #" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{F3A2CAFE-D999-47B2-8F66-908FB1558CAD}" name="Event Manager" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{64A085F6-E7D3-4DA3-AAC7-F81A271D4E49}" name="Mgr Email" dataDxfId="21"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{4F4945B9-D8C8-4B5B-B274-BAEF3F7791FF}" name="Venues" displayName="Venues" ref="A51:I60" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
+  <autoFilter ref="A51:I60" xr:uid="{4F4945B9-D8C8-4B5B-B274-BAEF3F7791FF}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{8F68947A-368E-455F-A420-8A157913600F}" name="Venue ID" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{18517D8A-8335-471A-9A4F-92CFD1D490A3}" name="Venue Location" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{AC36E7A4-59D8-4EB4-961D-CC44D1782FC2}" name="Location Address" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{28B6B0FE-FE2E-4BD3-A331-A92F5D15FE23}" name="Location City" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{A42BF559-1129-4CDC-A701-FE072F5CB789}" name="Location State" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{7920E893-3C56-4B26-9E09-1F6BC58EE365}" name="Location Zip" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{05646AE6-EDA6-4F59-ADBA-98B36E48CB89}" name="Venue Contact Name" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{8AF8FBAC-C93B-4381-A5E5-46183589BFF3}" name="Venue Email" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{C815A2FC-3014-436E-9DDC-12FDF7ADE851}" name="Venue Phone" dataDxfId="9"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{CC75FCEC-C214-4287-A6D2-30DB8AEBA7D7}" name="Events" displayName="Events" ref="A68:F79" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7" tableBorderDxfId="6">
+  <autoFilter ref="A68:F79" xr:uid="{CC75FCEC-C214-4287-A6D2-30DB8AEBA7D7}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{84A50774-3A30-491E-82FB-2EBF808DDBA5}" name="Event ID" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{AA3D1480-979F-4A04-8453-B588299D4E3D}" name="Event Name" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{84E7CCDE-8CD5-4D0F-8A5B-DC9E100DB8C5}" name="Event Date" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{591FF100-17F1-46A9-95B5-F59E40DC3C64}" name="Category Code" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{0C44F639-A7D1-48C6-A938-C0D700FFAFC8}" name="Employee #" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{8F411187-920F-4CF6-B25F-88A0BBC5124C}" name="Venue ID" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1290,29 +1708,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FA38BEC-78EC-44DC-83F3-AA711D021920}">
-  <dimension ref="A1:Q67"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Q82"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.28515625" customWidth="1"/>
-    <col min="2" max="2" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.140625" customWidth="1"/>
-    <col min="9" max="9" width="32.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="3" width="28.5703125" customWidth="1"/>
+    <col min="4" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="22.85546875" customWidth="1"/>
+    <col min="8" max="8" width="29.5703125" customWidth="1"/>
+    <col min="9" max="9" width="21" customWidth="1"/>
+    <col min="10" max="10" width="21.7109375" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.7109375" customWidth="1"/>
+    <col min="12" max="12" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="31.5703125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="30.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1320,63 +1735,63 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>113</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>103</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>104</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>105</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>107</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>106</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>90</v>
+        <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>91</v>
+        <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>92</v>
+        <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>93</v>
+        <v>12</v>
       </c>
       <c r="N1" t="s">
-        <v>114</v>
+        <v>13</v>
       </c>
       <c r="O1" t="s">
-        <v>96</v>
+        <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>94</v>
+        <v>15</v>
       </c>
       <c r="Q1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17">
       <c r="A2">
         <v>102</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E2">
         <v>7</v>
@@ -1385,51 +1800,51 @@
         <v>46095</v>
       </c>
       <c r="G2" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H2" t="s">
-        <v>108</v>
+        <v>21</v>
       </c>
       <c r="I2" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="J2" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="K2" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="L2" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="M2">
         <v>90026</v>
       </c>
       <c r="N2" t="s">
-        <v>116</v>
+        <v>26</v>
       </c>
       <c r="O2" t="s">
-        <v>98</v>
+        <v>27</v>
       </c>
       <c r="P2" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="Q2" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17">
       <c r="A3">
         <v>103</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="C3" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E3">
         <v>7</v>
@@ -1438,51 +1853,51 @@
         <v>46194</v>
       </c>
       <c r="G3" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H3" t="s">
-        <v>109</v>
+        <v>33</v>
       </c>
       <c r="I3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" t="s">
         <v>37</v>
-      </c>
-      <c r="J3" t="s">
-        <v>47</v>
-      </c>
-      <c r="K3" t="s">
-        <v>48</v>
-      </c>
-      <c r="L3" t="s">
-        <v>49</v>
       </c>
       <c r="M3">
         <v>78741</v>
       </c>
       <c r="N3" t="s">
-        <v>115</v>
+        <v>38</v>
       </c>
       <c r="O3" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="P3" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="Q3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17">
       <c r="A4">
         <v>104</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="E4">
         <v>2</v>
@@ -1491,51 +1906,51 @@
         <v>46115</v>
       </c>
       <c r="G4" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="H4" t="s">
-        <v>110</v>
+        <v>46</v>
       </c>
       <c r="I4" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="J4" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="K4" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="L4" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="M4">
         <v>90046</v>
       </c>
       <c r="N4" t="s">
-        <v>117</v>
+        <v>50</v>
       </c>
       <c r="O4" t="s">
-        <v>99</v>
+        <v>51</v>
       </c>
       <c r="P4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="Q4" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17">
       <c r="A5">
         <v>105</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="E5">
         <v>3</v>
@@ -1544,13 +1959,13 @@
         <v>46157</v>
       </c>
       <c r="G5" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H5" t="s">
-        <v>109</v>
+        <v>33</v>
       </c>
       <c r="I5" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="J5" t="s">
         <v>57</v>
@@ -1565,30 +1980,30 @@
         <v>60616</v>
       </c>
       <c r="N5" t="s">
-        <v>118</v>
+        <v>60</v>
       </c>
       <c r="O5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="P5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q5" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17">
       <c r="A6">
         <v>106</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>65</v>
       </c>
       <c r="D6" t="s">
-        <v>19</v>
+        <v>66</v>
       </c>
       <c r="E6">
         <v>6</v>
@@ -1597,51 +2012,51 @@
         <v>46109</v>
       </c>
       <c r="G6" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="H6" t="s">
-        <v>125</v>
+        <v>68</v>
       </c>
       <c r="I6" t="s">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="J6" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="K6" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="L6" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="M6">
         <v>10011</v>
       </c>
       <c r="N6" t="s">
-        <v>119</v>
+        <v>73</v>
       </c>
       <c r="O6" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="P6" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="Q6" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17">
       <c r="A7">
         <v>107</v>
       </c>
       <c r="B7" t="s">
-        <v>21</v>
+        <v>77</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>78</v>
       </c>
       <c r="E7">
         <v>4</v>
@@ -1650,13 +2065,13 @@
         <v>46130</v>
       </c>
       <c r="G7" t="s">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="H7" t="s">
-        <v>111</v>
+        <v>80</v>
       </c>
       <c r="I7" t="s">
-        <v>40</v>
+        <v>81</v>
       </c>
       <c r="J7" t="s">
         <v>57</v>
@@ -1671,30 +2086,30 @@
         <v>60616</v>
       </c>
       <c r="N7" t="s">
-        <v>118</v>
+        <v>60</v>
       </c>
       <c r="O7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="P7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="Q7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
       <c r="A8">
         <v>108</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>82</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>84</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -1703,51 +2118,51 @@
         <v>46144</v>
       </c>
       <c r="G8" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="H8" t="s">
-        <v>110</v>
+        <v>46</v>
       </c>
       <c r="I8" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="J8" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
       <c r="K8" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
       <c r="L8" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
       <c r="M8">
         <v>97214</v>
       </c>
       <c r="N8" t="s">
-        <v>120</v>
+        <v>88</v>
       </c>
       <c r="O8" t="s">
-        <v>72</v>
+        <v>89</v>
       </c>
       <c r="P8" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="Q8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17">
       <c r="A9">
         <v>109</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>92</v>
       </c>
       <c r="C9" t="s">
-        <v>28</v>
+        <v>93</v>
       </c>
       <c r="D9" t="s">
-        <v>16</v>
+        <v>56</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -1756,51 +2171,51 @@
         <v>46181</v>
       </c>
       <c r="G9" t="s">
-        <v>29</v>
+        <v>94</v>
       </c>
       <c r="H9" t="s">
-        <v>112</v>
+        <v>95</v>
       </c>
       <c r="I9" t="s">
-        <v>41</v>
+        <v>96</v>
       </c>
       <c r="J9" t="s">
-        <v>75</v>
+        <v>97</v>
       </c>
       <c r="K9" t="s">
-        <v>76</v>
+        <v>98</v>
       </c>
       <c r="L9" t="s">
-        <v>77</v>
+        <v>99</v>
       </c>
       <c r="M9">
         <v>48226</v>
       </c>
       <c r="N9" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="O9" t="s">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="P9" t="s">
-        <v>79</v>
+        <v>102</v>
       </c>
       <c r="Q9" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17">
       <c r="A10">
         <v>110</v>
       </c>
       <c r="B10" t="s">
-        <v>30</v>
+        <v>104</v>
       </c>
       <c r="C10" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="E10">
         <v>7</v>
@@ -1809,51 +2224,51 @@
         <v>46215</v>
       </c>
       <c r="G10" t="s">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H10" t="s">
-        <v>109</v>
+        <v>33</v>
       </c>
       <c r="I10" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="J10" t="s">
-        <v>42</v>
+        <v>23</v>
       </c>
       <c r="K10" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="L10" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="M10">
         <v>90026</v>
       </c>
       <c r="N10" t="s">
-        <v>116</v>
+        <v>26</v>
       </c>
       <c r="O10" t="s">
-        <v>98</v>
+        <v>27</v>
       </c>
       <c r="P10" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="Q10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17">
       <c r="A11">
         <v>111</v>
       </c>
       <c r="B11" t="s">
-        <v>31</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>106</v>
       </c>
       <c r="D11" t="s">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="E11">
         <v>2</v>
@@ -1862,51 +2277,51 @@
         <v>46102</v>
       </c>
       <c r="G11" t="s">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="H11" t="s">
-        <v>110</v>
+        <v>46</v>
       </c>
       <c r="I11" t="s">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="J11" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="K11" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="L11" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="M11">
         <v>10012</v>
       </c>
       <c r="N11" t="s">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="O11" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="P11" t="s">
-        <v>82</v>
+        <v>110</v>
       </c>
       <c r="Q11" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17">
       <c r="A12">
         <v>112</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>112</v>
       </c>
       <c r="C12" t="s">
-        <v>34</v>
+        <v>113</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>114</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -1915,74 +2330,782 @@
         <v>46137</v>
       </c>
       <c r="G12" t="s">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="H12" t="s">
-        <v>125</v>
+        <v>68</v>
       </c>
       <c r="I12" t="s">
-        <v>39</v>
+        <v>69</v>
       </c>
       <c r="J12" t="s">
-        <v>84</v>
+        <v>115</v>
       </c>
       <c r="K12" t="s">
-        <v>85</v>
+        <v>116</v>
       </c>
       <c r="L12" t="s">
-        <v>86</v>
+        <v>117</v>
       </c>
       <c r="M12">
         <v>33132</v>
       </c>
       <c r="N12" t="s">
+        <v>118</v>
+      </c>
+      <c r="O12" t="s">
+        <v>119</v>
+      </c>
+      <c r="P12" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" s="2" customFormat="1" thickBot="1"/>
+    <row r="16" spans="1:17" ht="18.75">
+      <c r="A16" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="B16" s="3"/>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" s="8">
+        <v>1</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" s="8">
+        <v>2</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" s="8">
+        <v>3</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" s="8">
+        <v>4</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" s="8">
+        <v>5</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" s="8">
+        <v>6</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" s="8">
+        <v>7</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="18.75">
+      <c r="A33" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="O12" t="s">
-        <v>87</v>
-      </c>
-      <c r="P12" t="s">
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="18.75">
+      <c r="A50" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D51" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="I51" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C52" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F52" s="9">
+        <v>10011</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="I52" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="C53" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F53" s="9">
+        <v>10012</v>
+      </c>
+      <c r="G53" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="I53" s="6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="E54" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="F54" s="9">
+        <v>60616</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="I54" s="6" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9">
+      <c r="A55" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D55" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="E55" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="F55" s="9">
+        <v>33132</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="I55" s="6" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9">
+      <c r="A56" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="B56" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C56" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D56" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="E56" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="F56" s="9">
+        <v>48226</v>
+      </c>
+      <c r="G56" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="H56" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="I56" s="6" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9">
+      <c r="A57" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="B57" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="C57" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="D57" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="E57" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F57" s="9">
+        <v>90046</v>
+      </c>
+      <c r="G57" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="H57" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="I57" s="6" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9">
+      <c r="A58" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="Q12" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="14" spans="1:17" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="15" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="B58" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="D58" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="E58" s="6" t="s">
+        <v>161</v>
+      </c>
+      <c r="F58" s="9">
+        <v>97214</v>
+      </c>
+      <c r="G58" s="6" t="s">
+        <v>162</v>
+      </c>
+      <c r="H58" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="I58" s="6" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9">
+      <c r="A59" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="D59" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="E59" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="F59" s="9">
+        <v>78741</v>
+      </c>
+      <c r="G59" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="H59" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="I59" s="6" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9">
+      <c r="A60" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B60" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C60" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="D60" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="E60" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F60" s="9">
+        <v>90026</v>
+      </c>
+      <c r="G60" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="H60" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="I60" s="6" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="18.75">
+      <c r="A67" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="B67" s="3"/>
+      <c r="C67" s="3"/>
+      <c r="D67" s="3"/>
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
+    </row>
+    <row r="68" spans="1:6">
+      <c r="A68" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="E68" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6">
+      <c r="A69" s="8">
+        <v>102</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C69" s="7">
+        <v>46095</v>
+      </c>
+      <c r="D69" s="8">
+        <v>7</v>
+      </c>
+      <c r="E69" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F69" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6">
+      <c r="A70" s="8">
+        <v>103</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C70" s="7">
+        <v>46194</v>
+      </c>
+      <c r="D70" s="8">
+        <v>7</v>
+      </c>
+      <c r="E70" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F70" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6">
+      <c r="A71" s="8">
+        <v>104</v>
+      </c>
+      <c r="B71" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C71" s="7">
+        <v>46115</v>
+      </c>
+      <c r="D71" s="8">
+        <v>2</v>
+      </c>
+      <c r="E71" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F71" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" s="8">
+        <v>105</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="C72" s="7">
+        <v>46157</v>
+      </c>
+      <c r="D72" s="8">
+        <v>3</v>
+      </c>
+      <c r="E72" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F72" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6">
+      <c r="A73" s="8">
+        <v>106</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="C73" s="7">
+        <v>46109</v>
+      </c>
+      <c r="D73" s="8">
+        <v>6</v>
+      </c>
+      <c r="E73" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F73" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6">
+      <c r="A74" s="8">
+        <v>107</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="C74" s="7">
+        <v>46130</v>
+      </c>
+      <c r="D74" s="8">
+        <v>4</v>
+      </c>
+      <c r="E74" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="F74" s="6" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6">
+      <c r="A75" s="8">
+        <v>108</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C75" s="7">
+        <v>46144</v>
+      </c>
+      <c r="D75" s="8">
+        <v>5</v>
+      </c>
+      <c r="E75" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F75" s="6" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6">
+      <c r="A76" s="8">
+        <v>109</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="C76" s="7">
+        <v>46181</v>
+      </c>
+      <c r="D76" s="8">
+        <v>3</v>
+      </c>
+      <c r="E76" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F76" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B16" s="3"/>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B33" s="3"/>
-    </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A50" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="B50" s="3"/>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A67" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="B67" s="3"/>
+    </row>
+    <row r="77" spans="1:6">
+      <c r="A77" s="8">
+        <v>110</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C77" s="7">
+        <v>46215</v>
+      </c>
+      <c r="D77" s="8">
+        <v>7</v>
+      </c>
+      <c r="E77" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F77" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6">
+      <c r="A78" s="8">
+        <v>111</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C78" s="7">
+        <v>46102</v>
+      </c>
+      <c r="D78" s="8">
+        <v>2</v>
+      </c>
+      <c r="E78" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F78" s="6" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6">
+      <c r="A79" s="8">
+        <v>112</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="C79" s="7">
+        <v>46137</v>
+      </c>
+      <c r="D79" s="8">
+        <v>1</v>
+      </c>
+      <c r="E79" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F79" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1">
+      <c r="A82" t="s">
+        <v>177</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="J19:J29">
     <sortCondition ref="J19:J29"/>
   </sortState>
+  <mergeCells count="4">
+    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A50:I50"/>
+    <mergeCell ref="A67:F67"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="4">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA5D0A6329BB324E86983B32928CFC2E" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d7eac4bce3bbb09c82bd908806be82e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xmlns:ns3="ced60a7f-99b1-48d2-b555-34851c8026ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb51570e5b7cb8bd524bc2df5324d4a3" ns2:_="" ns3:_="">
     <xsd:import namespace="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
@@ -2223,15 +3346,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2244,39 +3358,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6414E68-BBC1-4A96-B078-EF7EE95D29CE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
-    <ds:schemaRef ds:uri="ced60a7f-99b1-48d2-b555-34851c8026ae"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48FB9E6-6DE3-40FB-81F7-677295638F7C}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48FB9E6-6DE3-40FB-81F7-677295638F7C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6414E68-BBC1-4A96-B078-EF7EE95D29CE}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EE6EC55-B0E7-4ACE-A5DA-E03DCA4973DE}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="ced60a7f-99b1-48d2-b555-34851c8026ae"/>
-    <ds:schemaRef ds:uri="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EE6EC55-B0E7-4ACE-A5DA-E03DCA4973DE}"/>
 </file>
</xml_diff>